<commit_message>
Update Numbers clues, support image addresses, and set one-minute penalty
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -2,21 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1隐秘的见证" sheetId="1" r:id="R921ed7b28deb42db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2消失的龙" sheetId="3" r:id="R92d348d292a24256"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1碑影迷踪" sheetId="1" r:id="Rd729c030b38a4747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2消失的龙" sheetId="3" r:id="R4708b088fd5a4f39"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t xml:space="preserve">网址</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">提示词</x:t>
-  </x:si>
-</x:sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -48,11 +41,14 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="2">
+  <x:cellXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -259,159 +255,186 @@
   <x:cols>
     <x:col min="1" max="1" width="9" customWidth="1"/>
     <x:col min="2" max="2" width="42.83203125" style="1" customWidth="1"/>
+    <x:col min="3" max="3" width="31.110000610351562" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="17">
-      <x:c r="A1" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34">
+    <x:row r="1" ht="16" hidden="0" customHeight="1">
+      <x:c r="A1" t="str">
+        <x:v>网址</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="str">
+        <x:v>提示词</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>图片地址</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A2" t="str">
         <x:v>ch1-1</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="str">
+      <x:c r="B2" s="2" t="str">
         <x:v>日记中的古诗提到两处古迹的名字，有一处现已无存，请找到仍然存在的古迹名称，即为答案。</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="34">
+      <x:c r="C2"/>
+    </x:row>
+    <x:row r="3" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A3" t="str">
         <x:v>ch1-2-1</x:v>
       </x:c>
-      <x:c r="B3" s="1" t="str">
-        <x:v>请找到《皇都篇》碑文拓片，碑文末尾的落款纪年，与现场石碑基座束腰处的水兽数目，共同组成4位数字密码。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="34">
+      <x:c r="B3" s="2" t="str">
+        <x:v>请找到《皇都篇》碑文拓片。碑文末尾的落款纪年，与现场石碑基座束腰处的水兽数目，共同组成4位数字密码。</x:v>
+      </x:c>
+      <x:c r="C3"/>
+    </x:row>
+    <x:row r="4" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A4" t="str">
         <x:v>ch1-2-2</x:v>
       </x:c>
-      <x:c r="B4" s="1" t="str">
+      <x:c r="B4" s="2" t="str">
         <x:v>《皇都篇》碑文末尾的落款纪年，即为密码前两位；石碑基座束腰处水兽的数量，即为后两位。</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="34">
+      <x:c r="C4"/>
+    </x:row>
+    <x:row r="5" ht="45.599998474121094" hidden="0" customHeight="1">
       <x:c r="A5" t="str">
         <x:v>ch1-2-3</x:v>
       </x:c>
-      <x:c r="B5" s="1" t="str">
-        <x:v>水兽并不在碑身，而在石碑基座束腰处，不要遗漏任何一面。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="51">
+      <x:c r="B5" s="2" t="str">
+        <x:v>水兽并不在碑身，而在石碑基座束腰处，基座有四面，不要遗漏任何一面。
+</x:v>
+      </x:c>
+      <x:c r="C5"/>
+    </x:row>
+    <x:row r="6" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A6" t="str">
         <x:v>ch1-3-1</x:v>
       </x:c>
-      <x:c r="B6" s="1" t="str">
-        <x:v>在燕墩所在位置向北望去半里左右会看到一座位于中轴线上的古代建筑。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="34">
+      <x:c r="B6" s="2" t="str">
+        <x:v>《日下旧闻考》中，有一句话被用蓝线标记出来。这句话描述了燕墩和下一处地点的位置关系。 +</x:v>
+      </x:c>
+      <x:c r="C6"/>
+    </x:row>
+    <x:row r="7" ht="57.599998474121094" hidden="0" customHeight="1">
       <x:c r="A7" t="str">
         <x:v>ch1-3-2</x:v>
       </x:c>
-      <x:c r="B7" s="1" t="str">
-        <x:v>请你找到一张古代城门的手绘图，站在门城楼前，找出实物与图中不同之处，然后标出对应坐标数字</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="51">
+      <x:c r="B7" s="2" t="str">
+        <x:v>请将那幅城门楼的彩画与现场的城门楼进行比对。找到不同之后，你会发现这处不同所对应的数字坐标。 + +如遇城楼修缮，现场无法完成调查，请退出当前页面，点击「求助提示3」。</x:v>
+      </x:c>
+      <x:c r="C7"/>
+    </x:row>
+    <x:row r="8" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A8" t="str">
         <x:v>ch1-4-1</x:v>
       </x:c>
-      <x:c r="B8" s="1" t="str">
-        <x:v>永定门的位置在明信片上地图中已经标出，据此，找到图中那个奇怪图形的位置并前往</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="51">
+      <x:c r="B8" s="2" t="str">
+        <x:v>永定门的位置在其彩画背面的地图中已经标出，据此，找到图中那个红色符号的位置并前往。 +</x:v>
+      </x:c>
+      <x:c r="C8"/>
+    </x:row>
+    <x:row r="9" ht="43.20000076293945" hidden="0" customHeight="1">
       <x:c r="A9" t="str">
         <x:v>ch1-4-2</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="str">
-        <x:v>民信片背面是八大怪的雕塑，但是有几位没有道具，请到现场找找，并找到没有道具的雕塑的相应数字</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="34">
+      <x:c r="B9" s="2" t="str">
+        <x:v>你会发现，有一张明信片上绘有这座建筑，这是一座钟楼，但是明信片上的钟面缺失了，画面顶部的碎片正是缺失的钟面。每一个碎片都对应了一个数字。</x:v>
+      </x:c>
+      <x:c r="C9"/>
+    </x:row>
+    <x:row r="10" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A10" t="str">
         <x:v>ch1-5-1</x:v>
       </x:c>
-      <x:c r="B10" s="1" t="str">
-        <x:v>这个艺术殿堂就是天桥剧场，在天桥剧场的建筑上，有一个金灿灿的装饰雕塑。其中有一个芭蕾女孩</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="34">
+      <x:c r="B10" s="2" t="str">
+        <x:v>这个艺术殿堂就是天桥剧场。在天桥剧场的建筑上，有一个金灿灿的装饰雕塑，其中有一个芭蕾女孩。 +</x:v>
+      </x:c>
+      <x:c r="C10"/>
+    </x:row>
+    <x:row r="11" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A11" t="str">
         <x:v>ch1-5-2</x:v>
       </x:c>
-      <x:c r="B11" s="1" t="str">
-        <x:v>芭蕾女孩的头和两只腿，分别指向钟表上的三组数字。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="34">
+      <x:c r="B11" s="2" t="str">
+        <x:v>试着将芭蕾女孩的透卡，叠放在上一关的“四面钟”上。再看看她的头与双腿，指向了什么数字。</x:v>
+      </x:c>
+      <x:c r="C11"/>
+    </x:row>
+    <x:row r="12" ht="16" hidden="0" customHeight="1">
       <x:c r="A12" t="str">
         <x:v>ch1-6-1</x:v>
       </x:c>
-      <x:c r="B12" s="1" t="str">
-        <x:v>既然是和时间相关的建筑，那么它上面一定有看时间的工具。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="34">
+      <x:c r="B12" s="2" t="str">
+        <x:v>就在四面钟的西面，矗立着八大怪的雕塑 +</x:v>
+      </x:c>
+      <x:c r="C12"/>
+    </x:row>
+    <x:row r="13" ht="57.599998474121094" hidden="0" customHeight="1">
       <x:c r="A13" t="str">
         <x:v>ch1-6-2</x:v>
       </x:c>
-      <x:c r="B13" s="1" t="str">
-        <x:v>四面钟钟表上的表盘上的花纹是菱形组成，找出图片上不一样的花纹，他们所指的数字就是答案</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="51">
+      <x:c r="B13" s="2" t="str">
+        <x:v>找到那幅天桥盛景图。在这幅图的背面，有八大怪的残影。请将这些残影向正面折过来，拼合成完整的人物形象，就会出现一个汉字。请按照现场八个人从西向东的顺序，依次记录这八个字。</x:v>
+      </x:c>
+      <x:c r="C13"/>
+    </x:row>
+    <x:row r="14" ht="45.599998474121094" hidden="0" customHeight="1">
       <x:c r="A14" t="str">
         <x:v>ch1-7-1</x:v>
       </x:c>
-      <x:c r="B14" s="1" t="str">
-        <x:v>在地图中可以找到天桥位置。找到天桥，自然就找到石碑</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="68">
+      <x:c r="B14" s="2" t="str">
+        <x:v>请对照《天桥盛景图》，在现实中找到画中的天桥。石碑，就在它旁边。
+</x:v>
+      </x:c>
+      <x:c r="C14"/>
+    </x:row>
+    <x:row r="15" ht="88.80000305175781" hidden="0" customHeight="1">
       <x:c r="A15" t="str">
         <x:v>ch1-7-2</x:v>
       </x:c>
-      <x:c r="B15" s="1" t="str">
-        <x:v>你会发现碑文拓片边上有号码，那是碑文中文字所在顺序，请按照号码所出现的顺序找出16个字，然后读出。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="51">
+      <x:c r="B15" s="2" t="str">
+        <x:v>你会发现有一张《树影中的旧碑》的明信片，它的背面是碑文，但有些字被红色符号覆盖。请对照现场的石碑碑文，还原被覆盖的文字。 +
+再按照碑文下方红色符号从左至右的顺序，依次找出对应的文字，组成一条23字讯息。
+</x:v>
+      </x:c>
+      <x:c r="C15"/>
+    </x:row>
+    <x:row r="16" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A16" t="str">
         <x:v>ch1-8-1</x:v>
       </x:c>
-      <x:c r="B16" s="1" t="str">
-        <x:v>根据古文中“合字而得”的提示，把丝工，广由，分别组合成两个字，然后，文中所说“文末纪年之数”即是乾隆落款年份数字，它的乘数为两位数字。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="34">
+      <x:c r="B16" s="2" t="str">
+        <x:v>请开启调查资料中封存的*最终附件*中的《碑刻龙纹初考》，你会发现有六条龙纹改变了视线。</x:v>
+      </x:c>
+      <x:c r="C16"/>
+    </x:row>
+    <x:row r="17" ht="57.599998474121094" hidden="0" customHeight="1">
       <x:c r="A17" t="str">
         <x:v>ch1-8-2</x:v>
       </x:c>
-      <x:c r="B17" s="1" t="str">
-        <x:v>“左丝”意为左边是绞丝旁，“右工”意为右边是工字，二者左右组合即可。“广”为上顶，“由”为下基同理。</x:v>
-      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>在碑文的四周共有14条龙，其中有三组龙，每组两条，彼此相望。
+ +请用直线分别连接每对互相对望的两条龙的龙眼，当三对目光彼此相遇时，答案便会显现。</x:v>
+      </x:c>
+      <x:c r="C17"/>
     </x:row>
     <x:row r="18" ht="34">
-      <x:c r="A18" t="str">
-        <x:v>ch1-9-1</x:v>
-      </x:c>
-      <x:c r="B18" s="1" t="str">
-        <x:v>如果你仔细观察会发现，民信片上的龙纹和石碑上的龙纹有不同，</x:v>
-      </x:c>
+      <x:c r="A18"/>
+      <x:c r="B18" s="1"/>
+      <x:c r="C18"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>ch1-9-2</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>你会发现四条龙两两相望，以直线连接他们的视线，交汇之处，就是答案所在。</x:v>
-      </x:c>
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -421,14 +444,110 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <x:cols>
+    <x:col min="3" max="3" width="31.110000610351562" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" t="s">
-        <x:v>1</x:v>
-      </x:c>
+    <x:row r="1" ht="16" hidden="0" customHeight="1">
+      <x:c r="A1" t="str">
+        <x:v>网址</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="str">
+        <x:v>提示词</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>图片地址</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4"/>
+      <x:c r="B4"/>
+      <x:c r="C4"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5"/>
+      <x:c r="B5"/>
+      <x:c r="C5"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6"/>
+      <x:c r="B6"/>
+      <x:c r="C6"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7"/>
+      <x:c r="B7"/>
+      <x:c r="C7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8"/>
+      <x:c r="B8"/>
+      <x:c r="C8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9"/>
+      <x:c r="B9"/>
+      <x:c r="C9"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11"/>
+      <x:c r="B11"/>
+      <x:c r="C11"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add ch1-3-3 as standalone image clue
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1碑影迷踪" sheetId="1" r:id="Rd729c030b38a4747"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2消失的龙" sheetId="3" r:id="R4708b088fd5a4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1碑影迷踪" sheetId="1" r:id="R0d479c53517f482f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2消失的龙" sheetId="3" r:id="R3688fc072da748ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -327,108 +327,112 @@
       </x:c>
       <x:c r="C7"/>
     </x:row>
-    <x:row r="8" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="8" ht="16" hidden="0" customHeight="1">
       <x:c r="A8" t="str">
+        <x:v>ch1-3-3</x:v>
+      </x:c>
+      <x:c r="B8" s="2"/>
+      <x:c r="C8" t="str">
+        <x:v>images/ch1-3-3.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A9" t="str">
         <x:v>ch1-4-1</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="str">
+      <x:c r="B9" s="2" t="str">
         <x:v>永定门的位置在其彩画背面的地图中已经标出，据此，找到图中那个红色符号的位置并前往。  </x:v>
       </x:c>
-      <x:c r="C8"/>
-    </x:row>
-    <x:row r="9" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A9" t="str">
+      <x:c r="C9"/>
+    </x:row>
+    <x:row r="10" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A10" t="str">
         <x:v>ch1-4-2</x:v>
       </x:c>
-      <x:c r="B9" s="2" t="str">
+      <x:c r="B10" s="2" t="str">
         <x:v>你会发现，有一张明信片上绘有这座建筑，这是一座钟楼，但是明信片上的钟面缺失了，画面顶部的碎片正是缺失的钟面。每一个碎片都对应了一个数字。</x:v>
-      </x:c>
-      <x:c r="C9"/>
-    </x:row>
-    <x:row r="10" ht="28.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A10" t="str">
-        <x:v>ch1-5-1</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="str">
-        <x:v>这个艺术殿堂就是天桥剧场。在天桥剧场的建筑上，有一个金灿灿的装饰雕塑，其中有一个芭蕾女孩。 -</x:v>
       </x:c>
       <x:c r="C10"/>
     </x:row>
     <x:row r="11" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A11" t="str">
+        <x:v>ch1-5-1</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>这个艺术殿堂就是天桥剧场。在天桥剧场的建筑上，有一个金灿灿的装饰雕塑，其中有一个芭蕾女孩。 +</x:v>
+      </x:c>
+      <x:c r="C11"/>
+    </x:row>
+    <x:row r="12" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A12" t="str">
         <x:v>ch1-5-2</x:v>
       </x:c>
-      <x:c r="B11" s="2" t="str">
+      <x:c r="B12" s="2" t="str">
         <x:v>试着将芭蕾女孩的透卡，叠放在上一关的“四面钟”上。再看看她的头与双腿，指向了什么数字。</x:v>
       </x:c>
-      <x:c r="C11"/>
-    </x:row>
-    <x:row r="12" ht="16" hidden="0" customHeight="1">
-      <x:c r="A12" t="str">
+      <x:c r="C12"/>
+    </x:row>
+    <x:row r="13" ht="16" hidden="0" customHeight="1">
+      <x:c r="A13" t="str">
         <x:v>ch1-6-1</x:v>
       </x:c>
-      <x:c r="B12" s="2" t="str">
+      <x:c r="B13" s="2" t="str">
         <x:v>就在四面钟的西面，矗立着八大怪的雕塑  </x:v>
       </x:c>
-      <x:c r="C12"/>
-    </x:row>
-    <x:row r="13" ht="57.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A13" t="str">
+      <x:c r="C13"/>
+    </x:row>
+    <x:row r="14" ht="57.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A14" t="str">
         <x:v>ch1-6-2</x:v>
       </x:c>
-      <x:c r="B13" s="2" t="str">
+      <x:c r="B14" s="2" t="str">
         <x:v>找到那幅天桥盛景图。在这幅图的背面，有八大怪的残影。请将这些残影向正面折过来，拼合成完整的人物形象，就会出现一个汉字。请按照现场八个人从西向东的顺序，依次记录这八个字。</x:v>
       </x:c>
-      <x:c r="C13"/>
-    </x:row>
-    <x:row r="14" ht="45.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A14" t="str">
+      <x:c r="C14"/>
+    </x:row>
+    <x:row r="15" ht="45.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A15" t="str">
         <x:v>ch1-7-1</x:v>
       </x:c>
-      <x:c r="B14" s="2" t="str">
+      <x:c r="B15" s="2" t="str">
         <x:v>请对照《天桥盛景图》，在现实中找到画中的天桥。石碑，就在它旁边。
 </x:v>
       </x:c>
-      <x:c r="C14"/>
-    </x:row>
-    <x:row r="15" ht="88.80000305175781" hidden="0" customHeight="1">
-      <x:c r="A15" t="str">
+      <x:c r="C15"/>
+    </x:row>
+    <x:row r="16" ht="88.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A16" t="str">
         <x:v>ch1-7-2</x:v>
       </x:c>
-      <x:c r="B15" s="2" t="str">
+      <x:c r="B16" s="2" t="str">
         <x:v>你会发现有一张《树影中的旧碑》的明信片，它的背面是碑文，但有些字被红色符号覆盖。请对照现场的石碑碑文，还原被覆盖的文字。  
 再按照碑文下方红色符号从左至右的顺序，依次找出对应的文字，组成一条23字讯息。
 </x:v>
       </x:c>
-      <x:c r="C15"/>
-    </x:row>
-    <x:row r="16" ht="28.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A16" t="str">
+      <x:c r="C16"/>
+    </x:row>
+    <x:row r="17" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A17" t="str">
         <x:v>ch1-8-1</x:v>
       </x:c>
-      <x:c r="B16" s="2" t="str">
+      <x:c r="B17" s="2" t="str">
         <x:v>请开启调查资料中封存的*最终附件*中的《碑刻龙纹初考》，你会发现有六条龙纹改变了视线。</x:v>
       </x:c>
-      <x:c r="C16"/>
-    </x:row>
-    <x:row r="17" ht="57.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A17" t="str">
+      <x:c r="C17"/>
+    </x:row>
+    <x:row r="18" ht="57.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A18" t="str">
         <x:v>ch1-8-2</x:v>
       </x:c>
-      <x:c r="B17" s="2" t="str">
+      <x:c r="B18" s="1" t="str">
         <x:v>在碑文的四周共有14条龙，其中有三组龙，每组两条，彼此相望。
   请用直线分别连接每对互相对望的两条龙的龙眼，当三对目光彼此相遇时，答案便会显现。</x:v>
       </x:c>
-      <x:c r="C17"/>
-    </x:row>
-    <x:row r="18" ht="34">
-      <x:c r="A18"/>
-      <x:c r="B18" s="1"/>
       <x:c r="C18"/>
     </x:row>
     <x:row r="19">

</xml_diff>